<commit_message>
fix(kbsv): support test-orders source redirect in callback to prevent unwanted login redirect
</commit_message>
<xml_diff>
--- a/data/CPI_VNM.xlsx
+++ b/data/CPI_VNM.xlsx
@@ -5,7 +5,7 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\0. Luu_Thu Huyen\Nam 2026\CPI\Tháng 6.2026\0. CÔNG BỐ THÁNG 6.2026\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\1. CPI 2026\1. CHỐT THÁNG 7.2026\3. CÔNG BỐ THÁNG 7 NĂM 2026 03.8.2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="516" uniqueCount="238">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="517" uniqueCount="239">
   <si>
     <t>DATA_DOMAIN</t>
   </si>
@@ -739,6 +739,9 @@
   </si>
   <si>
     <t>2026-06</t>
+  </si>
+  <si>
+    <t>2026-07</t>
   </si>
 </sst>
 </file>
@@ -750,7 +753,7 @@
     <numFmt numFmtId="164" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="[$-409]mmm\-yy;@"/>
   </numFmts>
-  <fonts count="28">
+  <fonts count="28" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color indexed="8"/>
@@ -1261,7 +1264,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{44889A44-8645-4601-8977-B14930E482A0}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{44889A44-8645-4601-8977-B14930E482A0}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1591,7 +1594,7 @@
     <tabColor rgb="FFFFFF00"/>
   </sheetPr>
   <dimension ref="A1:WMB47"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.28515625" style="16" customWidth="1"/>
     <col min="2" max="2" width="40.28515625" style="16" customWidth="1"/>
@@ -1602,7 +1605,7 @@
     <col min="16069" max="16163" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:68 15881:15888" s="6" customFormat="1" ht="9.75" customHeight="1" thickBot="1">
+    <row r="1" spans="1:68 15881:15888" s="6" customFormat="1" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5"/>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -1612,7 +1615,7 @@
       <c r="WMA1" s="3"/>
       <c r="WMB1" s="3"/>
     </row>
-    <row r="2" spans="1:68 15881:15888" s="6" customFormat="1">
+    <row r="2" spans="1:68 15881:15888" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>21</v>
       </c>
@@ -1629,7 +1632,7 @@
       <c r="WMA2" s="3"/>
       <c r="WMB2" s="3"/>
     </row>
-    <row r="3" spans="1:68 15881:15888" s="6" customFormat="1">
+    <row r="3" spans="1:68 15881:15888" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
         <v>24</v>
       </c>
@@ -1646,7 +1649,7 @@
       <c r="WMA3" s="3"/>
       <c r="WMB3" s="3"/>
     </row>
-    <row r="4" spans="1:68 15881:15888" s="6" customFormat="1">
+    <row r="4" spans="1:68 15881:15888" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -1667,7 +1670,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:68 15881:15888" s="6" customFormat="1">
+    <row r="5" spans="1:68 15881:15888" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>1</v>
       </c>
@@ -1688,7 +1691,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:68 15881:15888" s="6" customFormat="1" ht="15.75" thickBot="1">
+    <row r="6" spans="1:68 15881:15888" s="6" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>2</v>
       </c>
@@ -1708,7 +1711,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:68 15881:15888" s="6" customFormat="1">
+    <row r="7" spans="1:68 15881:15888" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>4</v>
       </c>
@@ -1728,7 +1731,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:68 15881:15888" s="6" customFormat="1">
+    <row r="8" spans="1:68 15881:15888" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>3</v>
       </c>
@@ -1746,7 +1749,7 @@
       <c r="WMA8" s="3"/>
       <c r="WMB8" s="3"/>
     </row>
-    <row r="9" spans="1:68 15881:15888" s="6" customFormat="1" ht="15.75" thickBot="1">
+    <row r="9" spans="1:68 15881:15888" s="6" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>9</v>
       </c>
@@ -1762,14 +1765,14 @@
       <c r="WMA9" s="3"/>
       <c r="WMB9" s="3"/>
     </row>
-    <row r="10" spans="1:68 15881:15888" s="6" customFormat="1" ht="6.75" customHeight="1" thickBot="1">
+    <row r="10" spans="1:68 15881:15888" s="6" customFormat="1" ht="6.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="13"/>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
       <c r="WMA10" s="3"/>
       <c r="WMB10" s="3"/>
     </row>
-    <row r="11" spans="1:68 15881:15888" ht="15.75" thickBot="1">
+    <row r="11" spans="1:68 15881:15888" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
         <v>7</v>
       </c>
@@ -1975,7 +1978,7 @@
         <v>212</v>
       </c>
     </row>
-    <row r="12" spans="1:68 15881:15888" s="8" customFormat="1">
+    <row r="12" spans="1:68 15881:15888" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="20"/>
       <c r="B12" s="21" t="s">
         <v>43</v>
@@ -1990,7 +1993,7 @@
       <c r="WMA12" s="23"/>
       <c r="WMB12" s="23"/>
     </row>
-    <row r="13" spans="1:68 15881:15888">
+    <row r="13" spans="1:68 15881:15888" x14ac:dyDescent="0.25">
       <c r="A13" s="24" t="s">
         <v>19</v>
       </c>
@@ -2200,7 +2203,7 @@
       <c r="WMA13"/>
       <c r="WMB13"/>
     </row>
-    <row r="14" spans="1:68 15881:15888">
+    <row r="14" spans="1:68 15881:15888" x14ac:dyDescent="0.25">
       <c r="A14" s="24" t="s">
         <v>31</v>
       </c>
@@ -2410,7 +2413,7 @@
       <c r="WMA14"/>
       <c r="WMB14"/>
     </row>
-    <row r="15" spans="1:68 15881:15888">
+    <row r="15" spans="1:68 15881:15888" x14ac:dyDescent="0.25">
       <c r="A15" s="24" t="s">
         <v>88</v>
       </c>
@@ -2620,7 +2623,7 @@
       <c r="WMA15"/>
       <c r="WMB15"/>
     </row>
-    <row r="16" spans="1:68 15881:15888">
+    <row r="16" spans="1:68 15881:15888" x14ac:dyDescent="0.25">
       <c r="A16" s="24" t="s">
         <v>122</v>
       </c>
@@ -2830,7 +2833,7 @@
       <c r="WMA16"/>
       <c r="WMB16"/>
     </row>
-    <row r="17" spans="1:69 15881:15888">
+    <row r="17" spans="1:69 15881:15888" x14ac:dyDescent="0.25">
       <c r="A17" s="24" t="s">
         <v>87</v>
       </c>
@@ -3040,7 +3043,7 @@
       <c r="WMA17"/>
       <c r="WMB17"/>
     </row>
-    <row r="18" spans="1:69 15881:15888">
+    <row r="18" spans="1:69 15881:15888" x14ac:dyDescent="0.25">
       <c r="A18" s="24" t="s">
         <v>32</v>
       </c>
@@ -3250,7 +3253,7 @@
       <c r="WMA18"/>
       <c r="WMB18"/>
     </row>
-    <row r="19" spans="1:69 15881:15888">
+    <row r="19" spans="1:69 15881:15888" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
         <v>33</v>
       </c>
@@ -3460,7 +3463,7 @@
       <c r="WMA19"/>
       <c r="WMB19"/>
     </row>
-    <row r="20" spans="1:69 15881:15888" ht="30">
+    <row r="20" spans="1:69 15881:15888" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="24" t="s">
         <v>34</v>
       </c>
@@ -3670,7 +3673,7 @@
       <c r="WMA20"/>
       <c r="WMB20"/>
     </row>
-    <row r="21" spans="1:69 15881:15888">
+    <row r="21" spans="1:69 15881:15888" x14ac:dyDescent="0.25">
       <c r="A21" s="24" t="s">
         <v>35</v>
       </c>
@@ -3880,7 +3883,7 @@
       <c r="WMA21"/>
       <c r="WMB21"/>
     </row>
-    <row r="22" spans="1:69 15881:15888">
+    <row r="22" spans="1:69 15881:15888" x14ac:dyDescent="0.25">
       <c r="A22" s="24" t="s">
         <v>36</v>
       </c>
@@ -4090,7 +4093,7 @@
       <c r="WMA22"/>
       <c r="WMB22"/>
     </row>
-    <row r="23" spans="1:69 15881:15888">
+    <row r="23" spans="1:69 15881:15888" x14ac:dyDescent="0.25">
       <c r="A23" s="24" t="s">
         <v>121</v>
       </c>
@@ -4300,7 +4303,7 @@
       <c r="WMA23"/>
       <c r="WMB23"/>
     </row>
-    <row r="24" spans="1:69 15881:15888">
+    <row r="24" spans="1:69 15881:15888" x14ac:dyDescent="0.25">
       <c r="A24" s="24" t="s">
         <v>37</v>
       </c>
@@ -4510,7 +4513,7 @@
       <c r="WMA24"/>
       <c r="WMB24"/>
     </row>
-    <row r="25" spans="1:69 15881:15888" ht="30">
+    <row r="25" spans="1:69 15881:15888" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="24" t="s">
         <v>38</v>
       </c>
@@ -4720,7 +4723,7 @@
       <c r="WMA25"/>
       <c r="WMB25"/>
     </row>
-    <row r="26" spans="1:69 15881:15888">
+    <row r="26" spans="1:69 15881:15888" x14ac:dyDescent="0.25">
       <c r="A26" s="16" t="s">
         <v>40</v>
       </c>
@@ -4930,7 +4933,7 @@
       <c r="WMA26"/>
       <c r="WMB26"/>
     </row>
-    <row r="27" spans="1:69 15881:15888">
+    <row r="27" spans="1:69 15881:15888" x14ac:dyDescent="0.25">
       <c r="A27" s="16" t="s">
         <v>123</v>
       </c>
@@ -5141,7 +5144,7 @@
       <c r="WMA27"/>
       <c r="WMB27"/>
     </row>
-    <row r="28" spans="1:69 15881:15888">
+    <row r="28" spans="1:69 15881:15888" x14ac:dyDescent="0.25">
       <c r="A28" s="24" t="s">
         <v>39</v>
       </c>
@@ -5351,7 +5354,7 @@
       <c r="WMA28"/>
       <c r="WMB28"/>
     </row>
-    <row r="29" spans="1:69 15881:15888">
+    <row r="29" spans="1:69 15881:15888" x14ac:dyDescent="0.25">
       <c r="A29" s="24" t="s">
         <v>41</v>
       </c>
@@ -5561,7 +5564,7 @@
       <c r="WMA29"/>
       <c r="WMB29"/>
     </row>
-    <row r="30" spans="1:69 15881:15888" s="8" customFormat="1">
+    <row r="30" spans="1:69 15881:15888" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="20"/>
       <c r="B30" s="21" t="s">
         <v>44</v>
@@ -5586,7 +5589,7 @@
       <c r="WMA30" s="23"/>
       <c r="WMB30" s="23"/>
     </row>
-    <row r="31" spans="1:69 15881:15888">
+    <row r="31" spans="1:69 15881:15888" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
         <v>30</v>
       </c>
@@ -5792,7 +5795,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="32" spans="1:69 15881:15888">
+    <row r="32" spans="1:69 15881:15888" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
         <v>42</v>
       </c>
@@ -5998,7 +6001,7 @@
         <v>33.56</v>
       </c>
     </row>
-    <row r="33" spans="1:68 15887:15888">
+    <row r="33" spans="1:68 15887:15888" x14ac:dyDescent="0.25">
       <c r="A33" s="16" t="s">
         <v>104</v>
       </c>
@@ -6204,7 +6207,7 @@
         <v>3.67</v>
       </c>
     </row>
-    <row r="34" spans="1:68 15887:15888">
+    <row r="34" spans="1:68 15887:15888" x14ac:dyDescent="0.25">
       <c r="A34" s="16" t="s">
         <v>122</v>
       </c>
@@ -6410,7 +6413,7 @@
         <v>21.28</v>
       </c>
     </row>
-    <row r="35" spans="1:68 15887:15888">
+    <row r="35" spans="1:68 15887:15888" x14ac:dyDescent="0.25">
       <c r="A35" s="60" t="s">
         <v>170</v>
       </c>
@@ -6616,7 +6619,7 @@
         <v>8.61</v>
       </c>
     </row>
-    <row r="36" spans="1:68 15887:15888">
+    <row r="36" spans="1:68 15887:15888" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
         <v>105</v>
       </c>
@@ -6822,7 +6825,7 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="37" spans="1:68 15887:15888">
+    <row r="37" spans="1:68 15887:15888" x14ac:dyDescent="0.25">
       <c r="A37" s="16" t="s">
         <v>106</v>
       </c>
@@ -7028,7 +7031,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="38" spans="1:68 15887:15888" ht="45">
+    <row r="38" spans="1:68 15887:15888" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="16" t="s">
         <v>107</v>
       </c>
@@ -7234,7 +7237,7 @@
         <v>18.82</v>
       </c>
     </row>
-    <row r="39" spans="1:68 15887:15888">
+    <row r="39" spans="1:68 15887:15888" x14ac:dyDescent="0.25">
       <c r="A39" s="16" t="s">
         <v>108</v>
       </c>
@@ -7440,7 +7443,7 @@
         <v>6.74</v>
       </c>
     </row>
-    <row r="40" spans="1:68 15887:15888">
+    <row r="40" spans="1:68 15887:15888" x14ac:dyDescent="0.25">
       <c r="A40" s="16" t="s">
         <v>109</v>
       </c>
@@ -7646,7 +7649,7 @@
         <v>5.39</v>
       </c>
     </row>
-    <row r="41" spans="1:68 15887:15888">
+    <row r="41" spans="1:68 15887:15888" x14ac:dyDescent="0.25">
       <c r="A41" s="16" t="s">
         <v>110</v>
       </c>
@@ -7852,7 +7855,7 @@
         <v>9.67</v>
       </c>
     </row>
-    <row r="42" spans="1:68 15887:15888" ht="30">
+    <row r="42" spans="1:68 15887:15888" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="16" t="s">
         <v>111</v>
       </c>
@@ -8058,7 +8061,7 @@
         <v>3.14</v>
       </c>
     </row>
-    <row r="43" spans="1:68 15887:15888">
+    <row r="43" spans="1:68 15887:15888" x14ac:dyDescent="0.25">
       <c r="A43" s="16" t="s">
         <v>112</v>
       </c>
@@ -8264,7 +8267,7 @@
         <v>6.17</v>
       </c>
     </row>
-    <row r="44" spans="1:68 15887:15888" ht="30">
+    <row r="44" spans="1:68 15887:15888" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="16" t="s">
         <v>113</v>
       </c>
@@ -8470,7 +8473,7 @@
         <v>4.55</v>
       </c>
     </row>
-    <row r="45" spans="1:68 15887:15888" ht="30">
+    <row r="45" spans="1:68 15887:15888" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="16" t="s">
         <v>114</v>
       </c>
@@ -8676,7 +8679,7 @@
         <v>3.53</v>
       </c>
     </row>
-    <row r="46" spans="1:68 15887:15888" s="8" customFormat="1">
+    <row r="46" spans="1:68 15887:15888" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="20"/>
       <c r="B46" s="21" t="s">
         <v>115</v>
@@ -8698,7 +8701,7 @@
       <c r="WMA46" s="23"/>
       <c r="WMB46" s="23"/>
     </row>
-    <row r="47" spans="1:68 15887:15888">
+    <row r="47" spans="1:68 15887:15888" x14ac:dyDescent="0.25">
       <c r="A47" s="58" t="s">
         <v>120</v>
       </c>
@@ -8924,7 +8927,7 @@
     <tabColor rgb="FF92D050"/>
   </sheetPr>
   <dimension ref="A1:WJR47"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.28515625" style="16" customWidth="1"/>
     <col min="2" max="2" width="40.28515625" style="16" customWidth="1"/>
@@ -8935,7 +8938,7 @@
     <col min="16007" max="16101" width="9.140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16 15819:15826" s="6" customFormat="1" ht="9.75" customHeight="1" thickBot="1">
+    <row r="1" spans="1:16 15819:15826" s="6" customFormat="1" ht="9.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A1" s="5"/>
       <c r="B1" s="5"/>
       <c r="C1" s="5"/>
@@ -8943,7 +8946,7 @@
       <c r="WJQ1" s="3"/>
       <c r="WJR1" s="3"/>
     </row>
-    <row r="2" spans="1:16 15819:15826" s="6" customFormat="1">
+    <row r="2" spans="1:16 15819:15826" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="17" t="s">
         <v>21</v>
       </c>
@@ -8958,7 +8961,7 @@
       <c r="WJQ2" s="3"/>
       <c r="WJR2" s="3"/>
     </row>
-    <row r="3" spans="1:16 15819:15826" s="6" customFormat="1">
+    <row r="3" spans="1:16 15819:15826" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A3" s="17" t="s">
         <v>24</v>
       </c>
@@ -8973,7 +8976,7 @@
       <c r="WJQ3" s="3"/>
       <c r="WJR3" s="3"/>
     </row>
-    <row r="4" spans="1:16 15819:15826" s="6" customFormat="1">
+    <row r="4" spans="1:16 15819:15826" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>0</v>
       </c>
@@ -8992,7 +8995,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:16 15819:15826" s="6" customFormat="1">
+    <row r="5" spans="1:16 15819:15826" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>1</v>
       </c>
@@ -9011,7 +9014,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:16 15819:15826" s="6" customFormat="1" ht="15.75" thickBot="1">
+    <row r="6" spans="1:16 15819:15826" s="6" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="7" t="s">
         <v>2</v>
       </c>
@@ -9029,7 +9032,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:16 15819:15826" s="6" customFormat="1">
+    <row r="7" spans="1:16 15819:15826" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="9" t="s">
         <v>4</v>
       </c>
@@ -9047,7 +9050,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:16 15819:15826" s="6" customFormat="1">
+    <row r="8" spans="1:16 15819:15826" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>3</v>
       </c>
@@ -9063,7 +9066,7 @@
       <c r="WJQ8" s="3"/>
       <c r="WJR8" s="3"/>
     </row>
-    <row r="9" spans="1:16 15819:15826" s="6" customFormat="1" ht="15.75" thickBot="1">
+    <row r="9" spans="1:16 15819:15826" s="6" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>9</v>
       </c>
@@ -9077,12 +9080,12 @@
       <c r="WJQ9" s="3"/>
       <c r="WJR9" s="3"/>
     </row>
-    <row r="10" spans="1:16 15819:15826" s="6" customFormat="1" ht="6.75" customHeight="1" thickBot="1">
+    <row r="10" spans="1:16 15819:15826" s="6" customFormat="1" ht="6.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="13"/>
       <c r="WJQ10" s="3"/>
       <c r="WJR10" s="3"/>
     </row>
-    <row r="11" spans="1:16 15819:15826" ht="15.75" thickBot="1">
+    <row r="11" spans="1:16 15819:15826" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="14" t="s">
         <v>7</v>
       </c>
@@ -9123,8 +9126,11 @@
       <c r="N11" s="61" t="s">
         <v>237</v>
       </c>
-    </row>
-    <row r="12" spans="1:16 15819:15826" s="8" customFormat="1">
+      <c r="O11" s="61" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16 15819:15826" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A12" s="20"/>
       <c r="B12" s="21" t="s">
         <v>43</v>
@@ -9137,7 +9143,7 @@
       <c r="WJQ12" s="23"/>
       <c r="WJR12" s="23"/>
     </row>
-    <row r="13" spans="1:16 15819:15826">
+    <row r="13" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A13" s="24" t="s">
         <v>19</v>
       </c>
@@ -9179,6 +9185,9 @@
       </c>
       <c r="N13" s="52">
         <v>107.62753982213445</v>
+      </c>
+      <c r="O13" s="52">
+        <v>107.49591134093198</v>
       </c>
       <c r="P13" s="55"/>
       <c r="WJK13" s="4"/>
@@ -9186,7 +9195,7 @@
       <c r="WJQ13"/>
       <c r="WJR13"/>
     </row>
-    <row r="14" spans="1:16 15819:15826">
+    <row r="14" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A14" s="24" t="s">
         <v>31</v>
       </c>
@@ -9228,6 +9237,9 @@
       </c>
       <c r="N14" s="52">
         <v>107.22064570194172</v>
+      </c>
+      <c r="O14" s="52">
+        <v>107.14419738155624</v>
       </c>
       <c r="P14" s="55"/>
       <c r="WJK14" s="4"/>
@@ -9235,7 +9247,7 @@
       <c r="WJQ14"/>
       <c r="WJR14"/>
     </row>
-    <row r="15" spans="1:16 15819:15826">
+    <row r="15" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A15" s="24" t="s">
         <v>88</v>
       </c>
@@ -9277,6 +9289,9 @@
       </c>
       <c r="N15" s="52">
         <v>101.57458554584473</v>
+      </c>
+      <c r="O15" s="52">
+        <v>101.06620474518778</v>
       </c>
       <c r="P15" s="55"/>
       <c r="WJK15" s="4"/>
@@ -9284,7 +9299,7 @@
       <c r="WJQ15"/>
       <c r="WJR15"/>
     </row>
-    <row r="16" spans="1:16 15819:15826">
+    <row r="16" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A16" s="24" t="s">
         <v>122</v>
       </c>
@@ -9326,6 +9341,9 @@
       </c>
       <c r="N16" s="52">
         <v>106.98714603245749</v>
+      </c>
+      <c r="O16" s="52">
+        <v>106.91043624875221</v>
       </c>
       <c r="P16" s="55"/>
       <c r="WJK16" s="4"/>
@@ -9333,7 +9351,7 @@
       <c r="WJQ16"/>
       <c r="WJR16"/>
     </row>
-    <row r="17" spans="1:16 15819:15826">
+    <row r="17" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A17" s="24" t="s">
         <v>87</v>
       </c>
@@ -9375,6 +9393,9 @@
       </c>
       <c r="N17" s="52">
         <v>110.39564122765614</v>
+      </c>
+      <c r="O17" s="52">
+        <v>110.52866797533548</v>
       </c>
       <c r="P17" s="55"/>
       <c r="WJK17" s="4"/>
@@ -9382,7 +9403,7 @@
       <c r="WJQ17"/>
       <c r="WJR17"/>
     </row>
-    <row r="18" spans="1:16 15819:15826">
+    <row r="18" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A18" s="24" t="s">
         <v>32</v>
       </c>
@@ -9424,6 +9445,9 @@
       </c>
       <c r="N18" s="52">
         <v>105.70545426544894</v>
+      </c>
+      <c r="O18" s="52">
+        <v>105.89551267221822</v>
       </c>
       <c r="P18" s="55"/>
       <c r="WJK18" s="4"/>
@@ -9431,7 +9455,7 @@
       <c r="WJQ18"/>
       <c r="WJR18"/>
     </row>
-    <row r="19" spans="1:16 15819:15826">
+    <row r="19" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A19" s="24" t="s">
         <v>33</v>
       </c>
@@ -9473,6 +9497,9 @@
       </c>
       <c r="N19" s="52">
         <v>103.35334797059899</v>
+      </c>
+      <c r="O19" s="52">
+        <v>103.51375236664936</v>
       </c>
       <c r="P19" s="55"/>
       <c r="WJK19" s="4"/>
@@ -9480,7 +9507,7 @@
       <c r="WJQ19"/>
       <c r="WJR19"/>
     </row>
-    <row r="20" spans="1:16 15819:15826" ht="30">
+    <row r="20" spans="1:16 15819:15826" ht="30" x14ac:dyDescent="0.25">
       <c r="A20" s="24" t="s">
         <v>34</v>
       </c>
@@ -9522,6 +9549,9 @@
       </c>
       <c r="N20" s="52">
         <v>113.13256085180879</v>
+      </c>
+      <c r="O20" s="52">
+        <v>113.05348119177337</v>
       </c>
       <c r="P20" s="55"/>
       <c r="WJK20" s="4"/>
@@ -9529,7 +9559,7 @@
       <c r="WJQ20"/>
       <c r="WJR20"/>
     </row>
-    <row r="21" spans="1:16 15819:15826">
+    <row r="21" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A21" s="24" t="s">
         <v>35</v>
       </c>
@@ -9571,6 +9601,9 @@
       </c>
       <c r="N21" s="52">
         <v>104.96089822286751</v>
+      </c>
+      <c r="O21" s="52">
+        <v>105.11015262014044</v>
       </c>
       <c r="P21" s="55"/>
       <c r="WJK21" s="4"/>
@@ -9578,7 +9611,7 @@
       <c r="WJQ21"/>
       <c r="WJR21"/>
     </row>
-    <row r="22" spans="1:16 15819:15826">
+    <row r="22" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A22" s="24" t="s">
         <v>36</v>
       </c>
@@ -9620,6 +9653,9 @@
       </c>
       <c r="N22" s="52">
         <v>107.34849682018013</v>
+      </c>
+      <c r="O22" s="52">
+        <v>107.42879349580161</v>
       </c>
       <c r="P22" s="55"/>
       <c r="WJK22" s="4"/>
@@ -9627,7 +9663,7 @@
       <c r="WJQ22"/>
       <c r="WJR22"/>
     </row>
-    <row r="23" spans="1:16 15819:15826">
+    <row r="23" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A23" s="24" t="s">
         <v>121</v>
       </c>
@@ -9669,6 +9705,9 @@
       </c>
       <c r="N23" s="52">
         <v>109.41121404757543</v>
+      </c>
+      <c r="O23" s="52">
+        <v>109.43703509409066</v>
       </c>
       <c r="P23" s="55"/>
       <c r="WJK23" s="4"/>
@@ -9676,7 +9715,7 @@
       <c r="WJQ23"/>
       <c r="WJR23"/>
     </row>
-    <row r="24" spans="1:16 15819:15826">
+    <row r="24" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A24" s="24" t="s">
         <v>37</v>
       </c>
@@ -9718,6 +9757,9 @@
       </c>
       <c r="N24" s="52">
         <v>101.5223865651101</v>
+      </c>
+      <c r="O24" s="52">
+        <v>99.467878028191947</v>
       </c>
       <c r="P24" s="55"/>
       <c r="WJK24" s="4"/>
@@ -9725,7 +9767,7 @@
       <c r="WJQ24"/>
       <c r="WJR24"/>
     </row>
-    <row r="25" spans="1:16 15819:15826" ht="30">
+    <row r="25" spans="1:16 15819:15826" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="24" t="s">
         <v>38</v>
       </c>
@@ -9767,6 +9809,9 @@
       </c>
       <c r="N25" s="52">
         <v>100.51132747331572</v>
+      </c>
+      <c r="O25" s="52">
+        <v>100.61244186875386</v>
       </c>
       <c r="P25" s="55"/>
       <c r="WJK25" s="4"/>
@@ -9774,7 +9819,7 @@
       <c r="WJQ25"/>
       <c r="WJR25"/>
     </row>
-    <row r="26" spans="1:16 15819:15826">
+    <row r="26" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A26" s="16" t="s">
         <v>40</v>
       </c>
@@ -9816,6 +9861,9 @@
       </c>
       <c r="N26" s="52">
         <v>111.37274544106407</v>
+      </c>
+      <c r="O26" s="52">
+        <v>111.63825806619556</v>
       </c>
       <c r="P26" s="55"/>
       <c r="WJN26" s="4"/>
@@ -9823,7 +9871,7 @@
       <c r="WJQ26"/>
       <c r="WJR26"/>
     </row>
-    <row r="27" spans="1:16 15819:15826">
+    <row r="27" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A27" s="16" t="s">
         <v>123</v>
       </c>
@@ -9865,6 +9913,9 @@
       </c>
       <c r="N27" s="52">
         <v>112.60831240497782</v>
+      </c>
+      <c r="O27" s="52">
+        <v>112.93397564445303</v>
       </c>
       <c r="P27" s="55"/>
       <c r="WJN27" s="4"/>
@@ -9872,7 +9923,7 @@
       <c r="WJQ27"/>
       <c r="WJR27"/>
     </row>
-    <row r="28" spans="1:16 15819:15826">
+    <row r="28" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A28" s="24" t="s">
         <v>39</v>
       </c>
@@ -9914,6 +9965,9 @@
       </c>
       <c r="N28" s="52">
         <v>104.47640388022941</v>
+      </c>
+      <c r="O28" s="52">
+        <v>105.01978565681048</v>
       </c>
       <c r="P28" s="55"/>
       <c r="WJK28" s="4"/>
@@ -9921,7 +9975,7 @@
       <c r="WJQ28"/>
       <c r="WJR28"/>
     </row>
-    <row r="29" spans="1:16 15819:15826">
+    <row r="29" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A29" s="24" t="s">
         <v>41</v>
       </c>
@@ -9963,6 +10017,9 @@
       </c>
       <c r="N29" s="52">
         <v>109.04582387140415</v>
+      </c>
+      <c r="O29" s="52">
+        <v>111.18170442357334</v>
       </c>
       <c r="P29" s="55"/>
       <c r="WJK29" s="4"/>
@@ -9970,7 +10027,7 @@
       <c r="WJQ29"/>
       <c r="WJR29"/>
     </row>
-    <row r="30" spans="1:16 15819:15826" s="8" customFormat="1">
+    <row r="30" spans="1:16 15819:15826" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A30" s="20"/>
       <c r="B30" s="21" t="s">
         <v>44</v>
@@ -9984,7 +10041,7 @@
       <c r="WJQ30" s="23"/>
       <c r="WJR30" s="23"/>
     </row>
-    <row r="31" spans="1:16 15819:15826">
+    <row r="31" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A31" s="16" t="s">
         <v>30</v>
       </c>
@@ -10027,8 +10084,11 @@
       <c r="N31" s="52">
         <v>100</v>
       </c>
-    </row>
-    <row r="32" spans="1:16 15819:15826">
+      <c r="O31" s="52">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="32" spans="1:16 15819:15826" x14ac:dyDescent="0.25">
       <c r="A32" s="16" t="s">
         <v>42</v>
       </c>
@@ -10071,8 +10131,11 @@
       <c r="N32" s="52">
         <v>35.823212593699999</v>
       </c>
-    </row>
-    <row r="33" spans="1:14 15825:15826">
+      <c r="O32" s="52">
+        <v>35.823212593699999</v>
+      </c>
+    </row>
+    <row r="33" spans="1:15 15825:15826" x14ac:dyDescent="0.25">
       <c r="A33" s="16" t="s">
         <v>104</v>
       </c>
@@ -10115,8 +10178,11 @@
       <c r="N33" s="52">
         <v>4.1456756961000005</v>
       </c>
-    </row>
-    <row r="34" spans="1:14 15825:15826">
+      <c r="O33" s="52">
+        <v>4.1456756961000005</v>
+      </c>
+    </row>
+    <row r="34" spans="1:15 15825:15826" x14ac:dyDescent="0.25">
       <c r="A34" s="16" t="s">
         <v>122</v>
       </c>
@@ -10159,8 +10225,11 @@
       <c r="N34" s="52">
         <v>22.323992676</v>
       </c>
-    </row>
-    <row r="35" spans="1:14 15825:15826">
+      <c r="O34" s="52">
+        <v>22.323992676</v>
+      </c>
+    </row>
+    <row r="35" spans="1:15 15825:15826" x14ac:dyDescent="0.25">
       <c r="A35" s="60" t="s">
         <v>170</v>
       </c>
@@ -10203,8 +10272,11 @@
       <c r="N35" s="52">
         <v>9.3535442217</v>
       </c>
-    </row>
-    <row r="36" spans="1:14 15825:15826">
+      <c r="O35" s="52">
+        <v>9.3535442217</v>
+      </c>
+    </row>
+    <row r="36" spans="1:15 15825:15826" x14ac:dyDescent="0.25">
       <c r="A36" s="16" t="s">
         <v>105</v>
       </c>
@@ -10247,8 +10319,11 @@
       <c r="N36" s="52">
         <v>1.7513242057</v>
       </c>
-    </row>
-    <row r="37" spans="1:14 15825:15826">
+      <c r="O36" s="52">
+        <v>1.7513242057</v>
+      </c>
+    </row>
+    <row r="37" spans="1:15 15825:15826" x14ac:dyDescent="0.25">
       <c r="A37" s="16" t="s">
         <v>106</v>
       </c>
@@ -10291,8 +10366,11 @@
       <c r="N37" s="52">
         <v>3.5220945052000001</v>
       </c>
-    </row>
-    <row r="38" spans="1:14 15825:15826" ht="45">
+      <c r="O37" s="52">
+        <v>3.5220945052000001</v>
+      </c>
+    </row>
+    <row r="38" spans="1:15 15825:15826" ht="45" x14ac:dyDescent="0.25">
       <c r="A38" s="16" t="s">
         <v>107</v>
       </c>
@@ -10335,8 +10413,11 @@
       <c r="N38" s="52">
         <v>22.697484706599997</v>
       </c>
-    </row>
-    <row r="39" spans="1:14 15825:15826">
+      <c r="O38" s="52">
+        <v>22.697484706599997</v>
+      </c>
+    </row>
+    <row r="39" spans="1:15 15825:15826" x14ac:dyDescent="0.25">
       <c r="A39" s="16" t="s">
         <v>108</v>
       </c>
@@ -10379,8 +10460,11 @@
       <c r="N39" s="52">
         <v>5.1430623014000005</v>
       </c>
-    </row>
-    <row r="40" spans="1:14 15825:15826">
+      <c r="O39" s="52">
+        <v>5.1430623014000005</v>
+      </c>
+    </row>
+    <row r="40" spans="1:15 15825:15826" x14ac:dyDescent="0.25">
       <c r="A40" s="16" t="s">
         <v>109</v>
       </c>
@@ -10423,8 +10507,11 @@
       <c r="N40" s="52">
         <v>4.6611529854999993</v>
       </c>
-    </row>
-    <row r="41" spans="1:14 15825:15826">
+      <c r="O40" s="52">
+        <v>4.6611529854999993</v>
+      </c>
+    </row>
+    <row r="41" spans="1:15 15825:15826" x14ac:dyDescent="0.25">
       <c r="A41" s="16" t="s">
         <v>110</v>
       </c>
@@ -10467,8 +10554,11 @@
       <c r="N41" s="52">
         <v>9.9795999999999996</v>
       </c>
-    </row>
-    <row r="42" spans="1:14 15825:15826" ht="30">
+      <c r="O41" s="52">
+        <v>9.9795999999999996</v>
+      </c>
+    </row>
+    <row r="42" spans="1:15 15825:15826" ht="30" x14ac:dyDescent="0.25">
       <c r="A42" s="16" t="s">
         <v>111</v>
       </c>
@@ -10511,8 +10601,11 @@
       <c r="N42" s="52">
         <v>3.7356383262000001</v>
       </c>
-    </row>
-    <row r="43" spans="1:14 15825:15826">
+      <c r="O42" s="52">
+        <v>3.7356383262000001</v>
+      </c>
+    </row>
+    <row r="43" spans="1:15 15825:15826" x14ac:dyDescent="0.25">
       <c r="A43" s="16" t="s">
         <v>112</v>
       </c>
@@ -10555,8 +10648,11 @@
       <c r="N43" s="52">
         <v>5.9637911495000004</v>
       </c>
-    </row>
-    <row r="44" spans="1:14 15825:15826" ht="30">
+      <c r="O43" s="52">
+        <v>5.9637911495000004</v>
+      </c>
+    </row>
+    <row r="44" spans="1:15 15825:15826" ht="30" x14ac:dyDescent="0.25">
       <c r="A44" s="16" t="s">
         <v>113</v>
       </c>
@@ -10599,8 +10695,11 @@
       <c r="N44" s="52">
         <v>3.1426392262</v>
       </c>
-    </row>
-    <row r="45" spans="1:14 15825:15826" ht="30">
+      <c r="O44" s="52">
+        <v>3.1426392262</v>
+      </c>
+    </row>
+    <row r="45" spans="1:15 15825:15826" ht="30" x14ac:dyDescent="0.25">
       <c r="A45" s="16" t="s">
         <v>114</v>
       </c>
@@ -10643,8 +10742,11 @@
       <c r="N45" s="52">
         <v>3.58</v>
       </c>
-    </row>
-    <row r="46" spans="1:14 15825:15826" s="8" customFormat="1">
+      <c r="O45" s="52">
+        <v>3.58</v>
+      </c>
+    </row>
+    <row r="46" spans="1:15 15825:15826" s="8" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A46" s="20"/>
       <c r="B46" s="21" t="s">
         <v>115</v>
@@ -10657,7 +10759,7 @@
       <c r="WJQ46" s="23"/>
       <c r="WJR46" s="23"/>
     </row>
-    <row r="47" spans="1:14 15825:15826">
+    <row r="47" spans="1:15 15825:15826" x14ac:dyDescent="0.25">
       <c r="A47" s="58" t="s">
         <v>120</v>
       </c>
@@ -10699,6 +10801,9 @@
       </c>
       <c r="N47" s="52">
         <v>4.4957618993496817</v>
+      </c>
+      <c r="O47" s="52">
+        <v>4.6266401413648905</v>
       </c>
     </row>
   </sheetData>
@@ -10718,12 +10823,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:N82"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="34.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" ht="18.75">
+    <row r="1" spans="1:14" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A1" s="26" t="s">
         <v>45</v>
       </c>
@@ -10741,7 +10846,7 @@
       <c r="M1" s="25"/>
       <c r="N1" s="25"/>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="25"/>
       <c r="B3" s="25"/>
       <c r="C3" s="27" t="s">
@@ -10781,7 +10886,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="27">
         <v>2017</v>
       </c>
@@ -10825,7 +10930,7 @@
         <v>107.64</v>
       </c>
     </row>
-    <row r="5" spans="1:14">
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="25"/>
       <c r="B5" s="27" t="s">
         <v>58</v>
@@ -10867,7 +10972,7 @@
         <v>103.03</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="25"/>
       <c r="B6" s="27" t="s">
         <v>59</v>
@@ -10909,7 +11014,7 @@
         <v>105.15</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="25"/>
       <c r="B7" s="27" t="s">
         <v>60</v>
@@ -10951,7 +11056,7 @@
         <v>100.99</v>
       </c>
     </row>
-    <row r="8" spans="1:14">
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="25"/>
       <c r="B8" s="27" t="s">
         <v>61</v>
@@ -10993,7 +11098,7 @@
         <v>105.68</v>
       </c>
     </row>
-    <row r="9" spans="1:14">
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="25"/>
       <c r="B9" s="27" t="s">
         <v>62</v>
@@ -11035,7 +11140,7 @@
         <v>104.78</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="25"/>
       <c r="B10" s="27" t="s">
         <v>63</v>
@@ -11077,7 +11182,7 @@
         <v>107.12</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="25"/>
       <c r="B11" s="27" t="s">
         <v>64</v>
@@ -11119,7 +11224,7 @@
         <v>105.3</v>
       </c>
     </row>
-    <row r="12" spans="1:14">
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="25"/>
       <c r="B12" s="27" t="s">
         <v>65</v>
@@ -11161,7 +11266,7 @@
         <v>203.69</v>
       </c>
     </row>
-    <row r="13" spans="1:14">
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A13" s="25"/>
       <c r="B13" s="27" t="s">
         <v>27</v>
@@ -11203,7 +11308,7 @@
         <v>89.65</v>
       </c>
     </row>
-    <row r="14" spans="1:14">
+    <row r="14" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A14" s="25"/>
       <c r="B14" s="27" t="s">
         <v>66</v>
@@ -11245,7 +11350,7 @@
         <v>97.91</v>
       </c>
     </row>
-    <row r="15" spans="1:14">
+    <row r="15" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A15" s="25"/>
       <c r="B15" s="27" t="s">
         <v>28</v>
@@ -11287,7 +11392,7 @@
         <v>126.21</v>
       </c>
     </row>
-    <row r="16" spans="1:14">
+    <row r="16" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A16" s="25"/>
       <c r="B16" s="27" t="s">
         <v>67</v>
@@ -11329,7 +11434,7 @@
         <v>103.45</v>
       </c>
     </row>
-    <row r="17" spans="1:14">
+    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A17" s="25"/>
       <c r="B17" s="27" t="s">
         <v>68</v>
@@ -11371,7 +11476,7 @@
         <v>109.1</v>
       </c>
     </row>
-    <row r="18" spans="1:14">
+    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A18" s="25"/>
       <c r="B18" s="27" t="s">
         <v>69</v>
@@ -11413,7 +11518,7 @@
         <v>106.81</v>
       </c>
     </row>
-    <row r="19" spans="1:14">
+    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A19" s="25"/>
       <c r="B19" s="27" t="s">
         <v>70</v>
@@ -11455,7 +11560,7 @@
         <v>106.03</v>
       </c>
     </row>
-    <row r="20" spans="1:14">
+    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A20" s="27">
         <v>2016</v>
       </c>
@@ -11499,7 +11604,7 @@
         <v>104.91</v>
       </c>
     </row>
-    <row r="21" spans="1:14">
+    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A21" s="25"/>
       <c r="B21" s="27" t="s">
         <v>58</v>
@@ -11541,7 +11646,7 @@
         <v>104.92</v>
       </c>
     </row>
-    <row r="22" spans="1:14">
+    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A22" s="25"/>
       <c r="B22" s="27" t="s">
         <v>59</v>
@@ -11583,7 +11688,7 @@
         <v>101.97</v>
       </c>
     </row>
-    <row r="23" spans="1:14">
+    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A23" s="25"/>
       <c r="B23" s="27" t="s">
         <v>60</v>
@@ -11625,7 +11730,7 @@
         <v>105.11</v>
       </c>
     </row>
-    <row r="24" spans="1:14">
+    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A24" s="25"/>
       <c r="B24" s="27" t="s">
         <v>61</v>
@@ -11667,7 +11772,7 @@
         <v>104.25</v>
       </c>
     </row>
-    <row r="25" spans="1:14">
+    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A25" s="25"/>
       <c r="B25" s="27" t="s">
         <v>62</v>
@@ -11709,7 +11814,7 @@
         <v>103.6</v>
       </c>
     </row>
-    <row r="26" spans="1:14">
+    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A26" s="25"/>
       <c r="B26" s="27" t="s">
         <v>63</v>
@@ -11751,7 +11856,7 @@
         <v>102.34</v>
       </c>
     </row>
-    <row r="27" spans="1:14">
+    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A27" s="25"/>
       <c r="B27" s="27" t="s">
         <v>64</v>
@@ -11793,7 +11898,7 @@
         <v>104.17</v>
       </c>
     </row>
-    <row r="28" spans="1:14">
+    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A28" s="25"/>
       <c r="B28" s="27" t="s">
         <v>65</v>
@@ -11835,7 +11940,7 @@
         <v>159.38999999999999</v>
       </c>
     </row>
-    <row r="29" spans="1:14">
+    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A29" s="25"/>
       <c r="B29" s="27" t="s">
         <v>27</v>
@@ -11877,7 +11982,7 @@
         <v>84.54</v>
       </c>
     </row>
-    <row r="30" spans="1:14">
+    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A30" s="25"/>
       <c r="B30" s="27" t="s">
         <v>66</v>
@@ -11919,7 +12024,7 @@
         <v>98.36</v>
       </c>
     </row>
-    <row r="31" spans="1:14">
+    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A31" s="25"/>
       <c r="B31" s="27" t="s">
         <v>28</v>
@@ -11961,7 +12066,7 @@
         <v>117.64</v>
       </c>
     </row>
-    <row r="32" spans="1:14">
+    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A32" s="25"/>
       <c r="B32" s="27" t="s">
         <v>67</v>
@@ -12003,7 +12108,7 @@
         <v>102.66</v>
       </c>
     </row>
-    <row r="33" spans="1:14">
+    <row r="33" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A33" s="25"/>
       <c r="B33" s="27" t="s">
         <v>68</v>
@@ -12045,7 +12150,7 @@
         <v>106.61</v>
       </c>
     </row>
-    <row r="34" spans="1:14">
+    <row r="34" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A34" s="25"/>
       <c r="B34" s="27" t="s">
         <v>69</v>
@@ -12087,7 +12192,7 @@
         <v>101.98</v>
       </c>
     </row>
-    <row r="35" spans="1:14">
+    <row r="35" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A35" s="25"/>
       <c r="B35" s="27" t="s">
         <v>70</v>
@@ -12129,7 +12234,7 @@
         <v>106.08</v>
       </c>
     </row>
-    <row r="82" spans="1:1">
+    <row r="82" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A82" s="33" t="s">
         <v>119</v>
       </c>

</xml_diff>